<commit_message>
Update cadidate models, adding spring and summer precip as weather variables, calculate CWM
</commit_message>
<xml_diff>
--- a/00_rawdata/Cowichan IDE Trait Data Sheet.xlsx
+++ b/00_rawdata/Cowichan IDE Trait Data Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robin\Documents\School\Williams Lab\cowichan-diversity\00_rawdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD718A50-31A2-4EA2-A841-6FBAAA0C05F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B729DAD-440A-4619-A507-A2837B18951A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6777" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6770" uniqueCount="339">
   <si>
     <t>Trait Data Collection</t>
   </si>
@@ -544,19 +544,10 @@
     <t>growthform</t>
   </si>
   <si>
-    <t>photosynth</t>
-  </si>
-  <si>
-    <t>nfix</t>
-  </si>
-  <si>
     <t>duration</t>
   </si>
   <si>
     <t>nativity</t>
-  </si>
-  <si>
-    <t>no</t>
   </si>
   <si>
     <t>perennial</t>
@@ -566,9 +557,6 @@
   </si>
   <si>
     <t>forb</t>
-  </si>
-  <si>
-    <t>c3</t>
   </si>
   <si>
     <t>Poaceae</t>
@@ -638,9 +626,6 @@
   </si>
   <si>
     <t>Fabaceae</t>
-  </si>
-  <si>
-    <t>yes</t>
   </si>
   <si>
     <t>orchardgrass</t>
@@ -999,6 +984,105 @@
   <si>
     <t>ELGL_14_A</t>
   </si>
+  <si>
+    <t>genus</t>
+  </si>
+  <si>
+    <t>species_id</t>
+  </si>
+  <si>
+    <t>Amaryllidaceae</t>
+  </si>
+  <si>
+    <t>Allium_amplectens</t>
+  </si>
+  <si>
+    <t>Anthoxanthum_odoratum</t>
+  </si>
+  <si>
+    <t>Berberis_aquifolium</t>
+  </si>
+  <si>
+    <t>Bromus_carinatus</t>
+  </si>
+  <si>
+    <t>Bromus_hordeaceus</t>
+  </si>
+  <si>
+    <t>Bromus_sterilis</t>
+  </si>
+  <si>
+    <t>Camassia_quamash</t>
+  </si>
+  <si>
+    <t>Carex_inops</t>
+  </si>
+  <si>
+    <t>Cerastium_glomeratum</t>
+  </si>
+  <si>
+    <t>Claytonia_perfoliata</t>
+  </si>
+  <si>
+    <t>Dactylis_glomerata</t>
+  </si>
+  <si>
+    <t>Delphinium_menziesii</t>
+  </si>
+  <si>
+    <t>Elymus_glaucus</t>
+  </si>
+  <si>
+    <t>Erythronium_oregonum</t>
+  </si>
+  <si>
+    <t>Galium_aparine</t>
+  </si>
+  <si>
+    <t>Geranium_molle</t>
+  </si>
+  <si>
+    <t>Lathyrus_sphaericus</t>
+  </si>
+  <si>
+    <t>Lomatium_utriculatum</t>
+  </si>
+  <si>
+    <t>Melica_subulata</t>
+  </si>
+  <si>
+    <t>Nemophila_parviflora</t>
+  </si>
+  <si>
+    <t>Plectritis_congesta</t>
+  </si>
+  <si>
+    <t>Poa_pratensis</t>
+  </si>
+  <si>
+    <t>Primula_hendersonii</t>
+  </si>
+  <si>
+    <t>Ranunculus_occidentalis</t>
+  </si>
+  <si>
+    <t>Sanicula_crassicaulis</t>
+  </si>
+  <si>
+    <t>Symphoricarpos_albus</t>
+  </si>
+  <si>
+    <t>Valerianella_locusta</t>
+  </si>
+  <si>
+    <t>Veronica_arvensis</t>
+  </si>
+  <si>
+    <t>Vicia_hirsuta</t>
+  </si>
+  <si>
+    <t>Vicia_sativa</t>
+  </si>
 </sst>
 </file>
 
@@ -1009,7 +1093,7 @@
     <numFmt numFmtId="165" formatCode="m\-d"/>
     <numFmt numFmtId="166" formatCode="d\ mmmm\ yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1050,6 +1134,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1288,7 +1379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1367,6 +1458,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1677,19 +1769,19 @@
     </row>
     <row r="4" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -3074,21 +3166,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0579AFCC-ADF6-4BCA-94CD-AC203914402D}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>155</v>
+        <v>307</v>
       </c>
       <c r="B1" t="s">
         <v>156</v>
@@ -3105,774 +3196,645 @@
       <c r="F1" t="s">
         <v>160</v>
       </c>
-      <c r="G1" t="s">
-        <v>161</v>
-      </c>
-      <c r="H1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D2" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E2" t="s">
+        <v>161</v>
       </c>
       <c r="F2" t="s">
-        <v>163</v>
-      </c>
-      <c r="G2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" t="s">
         <v>167</v>
       </c>
-      <c r="F3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G3" t="s">
-        <v>164</v>
-      </c>
-      <c r="H3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D4" t="s">
-        <v>177</v>
+        <v>173</v>
+      </c>
+      <c r="E4" t="s">
+        <v>161</v>
       </c>
       <c r="F4" t="s">
-        <v>163</v>
-      </c>
-      <c r="G4" t="s">
-        <v>164</v>
-      </c>
-      <c r="H4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E5" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F5" t="s">
-        <v>163</v>
-      </c>
-      <c r="G5" t="s">
-        <v>164</v>
-      </c>
-      <c r="H5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D6" t="s">
-        <v>169</v>
+        <v>165</v>
+      </c>
+      <c r="E6" t="s">
+        <v>161</v>
       </c>
       <c r="F6" t="s">
-        <v>163</v>
-      </c>
-      <c r="G6" t="s">
-        <v>164</v>
-      </c>
-      <c r="H6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F7" t="s">
         <v>167</v>
       </c>
-      <c r="F7" t="s">
-        <v>163</v>
-      </c>
-      <c r="G7" t="s">
-        <v>170</v>
-      </c>
-      <c r="H7" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D8" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E8" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F8" t="s">
-        <v>163</v>
-      </c>
-      <c r="G8" t="s">
-        <v>164</v>
-      </c>
-      <c r="H8" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E9" t="s">
+        <v>161</v>
       </c>
       <c r="F9" t="s">
-        <v>163</v>
-      </c>
-      <c r="G9" t="s">
-        <v>164</v>
-      </c>
-      <c r="H9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C10" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E10" t="s">
         <v>166</v>
       </c>
       <c r="F10" t="s">
-        <v>163</v>
-      </c>
-      <c r="G10" t="s">
-        <v>170</v>
-      </c>
-      <c r="H10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C11" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E11" t="s">
         <v>166</v>
       </c>
-      <c r="E11" t="s">
-        <v>167</v>
-      </c>
       <c r="F11" t="s">
-        <v>163</v>
-      </c>
-      <c r="G11" t="s">
-        <v>170</v>
-      </c>
-      <c r="H11" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C12" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D12" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E12" t="s">
+        <v>161</v>
+      </c>
+      <c r="F12" t="s">
         <v>167</v>
       </c>
-      <c r="F12" t="s">
-        <v>163</v>
-      </c>
-      <c r="G12" t="s">
-        <v>164</v>
-      </c>
-      <c r="H12" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C13" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D13" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E13" t="s">
+        <v>161</v>
       </c>
       <c r="F13" t="s">
-        <v>163</v>
-      </c>
-      <c r="G13" t="s">
-        <v>164</v>
-      </c>
-      <c r="H13" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C14" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D14" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E14" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F14" t="s">
-        <v>163</v>
-      </c>
-      <c r="G14" t="s">
-        <v>164</v>
-      </c>
-      <c r="H14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C15" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E15" t="s">
+        <v>161</v>
       </c>
       <c r="F15" t="s">
-        <v>163</v>
-      </c>
-      <c r="G15" t="s">
-        <v>164</v>
-      </c>
-      <c r="H15" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C16" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D16" t="s">
+        <v>163</v>
+      </c>
+      <c r="E16" t="s">
         <v>166</v>
       </c>
       <c r="F16" t="s">
-        <v>163</v>
-      </c>
-      <c r="G16" t="s">
-        <v>170</v>
-      </c>
-      <c r="H16" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C17" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D17" t="s">
+        <v>163</v>
+      </c>
+      <c r="E17" t="s">
         <v>166</v>
       </c>
       <c r="F17" t="s">
-        <v>163</v>
-      </c>
-      <c r="G17" t="s">
-        <v>170</v>
-      </c>
-      <c r="H17" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C18" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E18" t="s">
         <v>166</v>
       </c>
       <c r="F18" t="s">
-        <v>191</v>
-      </c>
-      <c r="G18" t="s">
-        <v>170</v>
-      </c>
-      <c r="H18" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C19" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D19" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E19" t="s">
+        <v>161</v>
       </c>
       <c r="F19" t="s">
-        <v>163</v>
-      </c>
-      <c r="G19" t="s">
-        <v>164</v>
-      </c>
-      <c r="H19" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C20" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D20" t="s">
-        <v>169</v>
+        <v>165</v>
+      </c>
+      <c r="E20" t="s">
+        <v>161</v>
       </c>
       <c r="F20" t="s">
-        <v>207</v>
-      </c>
-      <c r="G20" t="s">
-        <v>164</v>
-      </c>
-      <c r="H20" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>91</v>
       </c>
       <c r="B21" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C21" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D21" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E21" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F21" t="s">
-        <v>163</v>
-      </c>
-      <c r="G21" t="s">
-        <v>164</v>
-      </c>
-      <c r="H21" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C22" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D22" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" t="s">
         <v>166</v>
       </c>
       <c r="F22" t="s">
-        <v>163</v>
-      </c>
-      <c r="G22" t="s">
-        <v>170</v>
-      </c>
-      <c r="H22" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C23" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D23" t="s">
+        <v>163</v>
+      </c>
+      <c r="E23" t="s">
         <v>166</v>
       </c>
       <c r="F23" t="s">
-        <v>163</v>
-      </c>
-      <c r="G23" t="s">
-        <v>170</v>
-      </c>
-      <c r="H23" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C24" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D24" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E24" t="s">
+        <v>161</v>
+      </c>
+      <c r="F24" t="s">
         <v>167</v>
       </c>
-      <c r="F24" t="s">
-        <v>163</v>
-      </c>
-      <c r="G24" t="s">
-        <v>164</v>
-      </c>
-      <c r="H24" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C25" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D25" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E25" t="s">
+        <v>161</v>
       </c>
       <c r="F25" t="s">
-        <v>163</v>
-      </c>
-      <c r="G25" t="s">
-        <v>164</v>
-      </c>
-      <c r="H25" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C26" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D26" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E26" t="s">
+        <v>161</v>
       </c>
       <c r="F26" t="s">
-        <v>163</v>
-      </c>
-      <c r="G26" t="s">
-        <v>164</v>
-      </c>
-      <c r="H26" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C27" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D27" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="E27" t="s">
+        <v>161</v>
       </c>
       <c r="F27" t="s">
-        <v>163</v>
-      </c>
-      <c r="G27" t="s">
-        <v>164</v>
-      </c>
-      <c r="H27" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C28" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D28" t="s">
-        <v>177</v>
+        <v>173</v>
+      </c>
+      <c r="E28" t="s">
+        <v>161</v>
       </c>
       <c r="F28" t="s">
-        <v>163</v>
-      </c>
-      <c r="G28" t="s">
-        <v>164</v>
-      </c>
-      <c r="H28" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C29" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D29" t="s">
+        <v>163</v>
+      </c>
+      <c r="E29" t="s">
         <v>166</v>
       </c>
       <c r="F29" t="s">
-        <v>163</v>
-      </c>
-      <c r="G29" t="s">
-        <v>170</v>
-      </c>
-      <c r="H29" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C30" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D30" t="s">
+        <v>163</v>
+      </c>
+      <c r="E30" t="s">
         <v>166</v>
       </c>
       <c r="F30" t="s">
-        <v>163</v>
-      </c>
-      <c r="G30" t="s">
-        <v>170</v>
-      </c>
-      <c r="H30" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>58</v>
       </c>
       <c r="B31" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C31" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D31" t="s">
+        <v>163</v>
+      </c>
+      <c r="E31" t="s">
         <v>166</v>
       </c>
       <c r="F31" t="s">
-        <v>191</v>
-      </c>
-      <c r="G31" t="s">
-        <v>170</v>
-      </c>
-      <c r="H31" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C32" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D32" t="s">
+        <v>163</v>
+      </c>
+      <c r="E32" t="s">
         <v>166</v>
       </c>
       <c r="F32" t="s">
-        <v>191</v>
-      </c>
-      <c r="G32" t="s">
-        <v>170</v>
-      </c>
-      <c r="H32" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>101</v>
       </c>
       <c r="B33" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D33" t="s">
-        <v>169</v>
+        <v>165</v>
+      </c>
+      <c r="E33" t="s">
+        <v>166</v>
       </c>
       <c r="F33" t="s">
-        <v>207</v>
-      </c>
-      <c r="G33" t="s">
-        <v>170</v>
-      </c>
-      <c r="H33" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -3887,371 +3849,482 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6659E37C-A85F-4E70-9B5F-7C39381BB3CC}">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>307</v>
       </c>
       <c r="B1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>309</v>
+      </c>
+      <c r="C2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>310</v>
+      </c>
+      <c r="C3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>311</v>
+      </c>
+      <c r="C4" t="s">
+        <v>224</v>
+      </c>
+      <c r="D4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>312</v>
+      </c>
+      <c r="C5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>313</v>
+      </c>
+      <c r="C6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="C8" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>316</v>
+      </c>
+      <c r="C9" t="s">
         <v>227</v>
       </c>
-      <c r="C1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="D9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="36" t="s">
+        <v>317</v>
+      </c>
+      <c r="C10" t="s">
         <v>228</v>
       </c>
-      <c r="C2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" t="s">
         <v>229</v>
       </c>
-      <c r="C3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D11" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="36" t="s">
+        <v>319</v>
+      </c>
+      <c r="C12" t="s">
         <v>230</v>
       </c>
-      <c r="C4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>230</v>
-      </c>
-      <c r="C5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="D12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="36" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" t="s">
         <v>231</v>
       </c>
-      <c r="C7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="D13" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>321</v>
+      </c>
+      <c r="C14" t="s">
         <v>232</v>
       </c>
-      <c r="C8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="D14" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>322</v>
+      </c>
+      <c r="C15" t="s">
         <v>233</v>
       </c>
-      <c r="C9" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="D15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>323</v>
+      </c>
+      <c r="C16" t="s">
         <v>234</v>
       </c>
-      <c r="C10" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="D16" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>324</v>
+      </c>
+      <c r="C17" t="s">
         <v>235</v>
       </c>
-      <c r="C11" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="D17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="36" t="s">
+        <v>325</v>
+      </c>
+      <c r="C18" t="s">
         <v>236</v>
       </c>
-      <c r="C12" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="D18" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="C19" t="s">
         <v>237</v>
       </c>
-      <c r="C13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="D19" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" t="s">
         <v>238</v>
       </c>
-      <c r="C14" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C20" t="s">
+        <v>238</v>
+      </c>
+      <c r="D20" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>327</v>
+      </c>
+      <c r="C21" t="s">
         <v>239</v>
       </c>
-      <c r="C15" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="D21" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>328</v>
+      </c>
+      <c r="C22" t="s">
         <v>240</v>
       </c>
-      <c r="C16" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="D22" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>329</v>
+      </c>
+      <c r="C23" t="s">
         <v>241</v>
       </c>
-      <c r="C17" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="D23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="36" t="s">
+        <v>330</v>
+      </c>
+      <c r="C24" t="s">
         <v>242</v>
       </c>
-      <c r="C18" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="D24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="36" t="s">
+        <v>331</v>
+      </c>
+      <c r="C25" t="s">
         <v>243</v>
       </c>
-      <c r="B19" t="s">
-        <v>243</v>
-      </c>
-      <c r="C19" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="D25" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>332</v>
+      </c>
+      <c r="C26" t="s">
         <v>244</v>
       </c>
-      <c r="C20" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="D26" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="36" t="s">
+        <v>333</v>
+      </c>
+      <c r="C27" t="s">
         <v>245</v>
       </c>
-      <c r="C21" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="D27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="36" t="s">
+        <v>334</v>
+      </c>
+      <c r="C28" t="s">
         <v>246</v>
       </c>
-      <c r="C22" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="D28" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="36" t="s">
+        <v>335</v>
+      </c>
+      <c r="C29" t="s">
         <v>247</v>
       </c>
-      <c r="C23" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="D29" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="36" t="s">
+        <v>336</v>
+      </c>
+      <c r="C30" t="s">
         <v>248</v>
       </c>
-      <c r="C24" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="D30" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>337</v>
+      </c>
+      <c r="C31" t="s">
         <v>249</v>
       </c>
-      <c r="C25" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="D31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>338</v>
+      </c>
+      <c r="C32" t="s">
+        <v>249</v>
+      </c>
+      <c r="D32" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" t="s">
         <v>250</v>
       </c>
-      <c r="C26" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" t="s">
-        <v>251</v>
-      </c>
-      <c r="C27" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" t="s">
-        <v>252</v>
-      </c>
-      <c r="C28" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" t="s">
-        <v>253</v>
-      </c>
-      <c r="C29" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>57</v>
-      </c>
-      <c r="B30" t="s">
-        <v>254</v>
-      </c>
-      <c r="C30" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" t="s">
-        <v>254</v>
-      </c>
-      <c r="C31" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>255</v>
-      </c>
-      <c r="B32" t="s">
-        <v>255</v>
-      </c>
-      <c r="C32" t="s">
-        <v>168</v>
+      <c r="C33" t="s">
+        <v>250</v>
+      </c>
+      <c r="D33" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:C32">
-    <sortCondition ref="A1:A32"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:D33">
+    <sortCondition ref="B2:B33"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4275,7 +4348,7 @@
         <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>307</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>151</v>
@@ -11820,7 +11893,7 @@
         <v>144</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>155</v>
+        <v>307</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>103</v>
@@ -11841,7 +11914,7 @@
         <v>146</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="K1" s="27" t="s">
         <v>16</v>
@@ -39547,24 +39620,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="34" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C1" s="34" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="D1" s="34" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="E1" s="34" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="34" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B2" s="34">
         <v>2.66</v>
@@ -39581,7 +39654,7 @@
     </row>
     <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="34" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B3" s="34">
         <v>2.2000000000000002</v>
@@ -39598,7 +39671,7 @@
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="34" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B4" s="34">
         <v>2.29</v>
@@ -39615,7 +39688,7 @@
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="34" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B5" s="35">
         <v>2.83</v>
@@ -39632,7 +39705,7 @@
     </row>
     <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="34" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B6" s="34">
         <v>2.4900000000000002</v>
@@ -39649,7 +39722,7 @@
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="34" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B7" s="34">
         <v>2.04</v>
@@ -39666,7 +39739,7 @@
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="34" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B8" s="34">
         <v>2.42</v>
@@ -39683,7 +39756,7 @@
     </row>
     <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="34" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B9" s="34">
         <v>2.77</v>
@@ -39700,7 +39773,7 @@
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="34" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B10" s="34">
         <v>2.19</v>
@@ -39717,7 +39790,7 @@
     </row>
     <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="34" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B11" s="34">
         <v>2.69</v>
@@ -39734,7 +39807,7 @@
     </row>
     <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="34" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B12" s="35">
         <v>2.89</v>
@@ -39751,7 +39824,7 @@
     </row>
     <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="34" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B13" s="35">
         <v>2.81</v>
@@ -39768,7 +39841,7 @@
     </row>
     <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="34" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B14" s="34">
         <v>2.09</v>
@@ -39785,7 +39858,7 @@
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="34" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B15" s="34">
         <v>2.54</v>
@@ -39802,7 +39875,7 @@
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="34" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B16" s="34">
         <v>2.1800000000000002</v>
@@ -39819,7 +39892,7 @@
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="34" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B17" s="34">
         <v>2.92</v>
@@ -39836,7 +39909,7 @@
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="34" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B18" s="34">
         <v>2.57</v>
@@ -39853,7 +39926,7 @@
     </row>
     <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="34" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B19" s="34">
         <v>2.93</v>
@@ -39870,7 +39943,7 @@
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="34" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B20" s="34">
         <v>2.65</v>
@@ -39887,7 +39960,7 @@
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="34" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B21" s="34">
         <v>2.37</v>
@@ -39904,7 +39977,7 @@
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="34" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B22" s="34">
         <v>2.2200000000000002</v>
@@ -39921,7 +39994,7 @@
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="34" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B23" s="34">
         <v>2.29</v>
@@ -39938,7 +40011,7 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="34" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B24" s="34">
         <v>2.42</v>
@@ -39955,7 +40028,7 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="34" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B25" s="34">
         <v>2.58</v>
@@ -39972,7 +40045,7 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="34" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B26" s="34">
         <v>2.44</v>
@@ -39989,7 +40062,7 @@
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="34" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B27" s="34">
         <v>2.85</v>
@@ -40006,7 +40079,7 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="34" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B28" s="34">
         <v>2.4900000000000002</v>
@@ -40023,7 +40096,7 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="34" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B29" s="34">
         <v>2.4500000000000002</v>
@@ -40040,7 +40113,7 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="34" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B30" s="34">
         <v>2.1</v>
@@ -40057,7 +40130,7 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="34" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B31" s="34">
         <v>2.19</v>
@@ -40074,7 +40147,7 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="34" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B32" s="34">
         <v>2.95</v>
@@ -40091,7 +40164,7 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="34" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B33" s="34">
         <v>2.35</v>
@@ -40108,7 +40181,7 @@
     </row>
     <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="34" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B34" s="34">
         <v>2.25</v>
@@ -40125,7 +40198,7 @@
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="34" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B35" s="34">
         <v>2.52</v>
@@ -40142,7 +40215,7 @@
     </row>
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="34" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B36" s="34">
         <v>2.91</v>
@@ -40159,7 +40232,7 @@
     </row>
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="34" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B37" s="34">
         <v>2.57</v>
@@ -40176,7 +40249,7 @@
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="34" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B38" s="34">
         <v>2.23</v>
@@ -40193,7 +40266,7 @@
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="34" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B39" s="34">
         <v>2.73</v>
@@ -40210,7 +40283,7 @@
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="34" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B40" s="34">
         <v>2.21</v>
@@ -40227,7 +40300,7 @@
     </row>
     <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="34" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B41" s="34">
         <v>2.25</v>
@@ -40244,7 +40317,7 @@
     </row>
     <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="34" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B42" s="34">
         <v>2.2200000000000002</v>
@@ -40261,7 +40334,7 @@
     </row>
     <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="34" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B43" s="34">
         <v>2.7</v>
@@ -40278,7 +40351,7 @@
     </row>
     <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="34" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B44" s="34">
         <v>2.21</v>
@@ -40295,7 +40368,7 @@
     </row>
     <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="34" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B45" s="34">
         <v>2.67</v>
@@ -40312,7 +40385,7 @@
     </row>
     <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="34" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B46" s="34">
         <v>2.97</v>
@@ -40329,7 +40402,7 @@
     </row>
     <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="34" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B47" s="34">
         <v>2.6</v>
@@ -40346,7 +40419,7 @@
     </row>
     <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="34" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B48" s="35">
         <v>2.7</v>

</xml_diff>